<commit_message>
fix(property): start additional rate at 125,140 total income in landlordTax
HIGHER_RATE_LIMIT was PA_TAPER_END - PERSONAL_ALLOWANCE = 112,570 in
taxable-income terms, starting the 45% band a full allowance early once
the PA tapers and overstating tax by up to 628.50. Replace with
ADDITIONAL_RATE_GROSS_THRESHOLD (125,140 total income) converted onto
the taxable axis via additionalRateLimitTaxable(pa), in both incomeTaxOn
and the computePortfolio band split.

- builder: Rates sheet row + bandedTaxFormula use AddlThreshold with the
  same taxable-axis conversion; xlsx regenerated (byte-stable build)
- golden: add taper-zone scenario (140k total income) that fails on the
  old threshold; both scenarios pass 8/8
- 2027 blog: correct rate table to 125,140 and recompute the Priya
  worked example with the PA taper (verified by hand)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Property/web/public/resources/landlord-essentials/landlord-essentials-model.xlsx
+++ b/Property/web/public/resources/landlord-essentials/landlord-essentials-model.xlsx
@@ -26,7 +26,7 @@
     <definedName name="PA_TaperStart">Rates!$B$11</definedName>
     <definedName name="PA_TaperEnd">Rates!$B$12</definedName>
     <definedName name="BasicLimit">Rates!$B$13</definedName>
-    <definedName name="HigherLimit">Rates!$B$14</definedName>
+    <definedName name="AddlThreshold">Rates!$B$14</definedName>
     <definedName name="PropAllowance">Rates!$B$15</definedName>
     <definedName name="In_Other">'Your figures'!$B$3</definedName>
     <definedName name="In_Year">'Your figures'!$B$4</definedName>
@@ -94,7 +94,7 @@
     <t>Top of basic-rate band — taxable income (£)</t>
   </si>
   <si>
-    <t>Top of higher-rate band — taxable income (£)</t>
+    <t>Additional-rate threshold — total income (£)</t>
   </si>
   <si>
     <t>Property allowance (£)</t>
@@ -874,7 +874,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="5">
-        <v>112570</v>
+        <v>125140</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -1182,7 +1182,7 @@
         <v>41</v>
       </c>
       <c r="B22" s="11">
-        <f>MIN(MAX(0,IncWith-PA_With),BasicLimit)*BasicRate+MIN(MAX(0,MAX(0,IncWith-PA_With)-BasicLimit),HigherLimit-BasicLimit)*HigherRate+MAX(0,MAX(0,IncWith-PA_With)-HigherLimit)*AddlRate</f>
+        <f>MIN(MAX(0,IncWith-PA_With),BasicLimit)*BasicRate+MIN(MAX(0,MAX(0,IncWith-PA_With)-BasicLimit),MAX(BasicLimit,AddlThreshold-PA_With)-BasicLimit)*HigherRate+MAX(0,MAX(0,IncWith-PA_With)-MAX(BasicLimit,AddlThreshold-PA_With))*AddlRate</f>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -1190,7 +1190,7 @@
         <v>42</v>
       </c>
       <c r="B23" s="11">
-        <f>MIN(MAX(0,In_Other-PA_Other),BasicLimit)*BasicRate+MIN(MAX(0,MAX(0,In_Other-PA_Other)-BasicLimit),HigherLimit-BasicLimit)*HigherRate+MAX(0,MAX(0,In_Other-PA_Other)-HigherLimit)*AddlRate</f>
+        <f>MIN(MAX(0,In_Other-PA_Other),BasicLimit)*BasicRate+MIN(MAX(0,MAX(0,In_Other-PA_Other)-BasicLimit),MAX(BasicLimit,AddlThreshold-PA_Other)-BasicLimit)*HigherRate+MAX(0,MAX(0,In_Other-PA_Other)-MAX(BasicLimit,AddlThreshold-PA_Other))*AddlRate</f>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>